<commit_message>
test de relation des langages
</commit_message>
<xml_diff>
--- a/data/SOMIDA_DAF_2025.xlsx
+++ b/data/SOMIDA_DAF_2025.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Documents/DIX Y/SOMIDA/SIMP/sxmxdxSimp/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85C60343-9D7C-914B-9945-307BA4D694C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A984C191-20B9-2347-836B-61880A260435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16100" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -939,6 +939,24 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -953,24 +971,6 @@
     </xf>
     <xf numFmtId="166" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1185,7 +1185,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="26.1640625" customWidth="1"/>
@@ -1201,7 +1201,7 @@
       <c r="C1" s="33"/>
       <c r="D1" s="33"/>
     </row>
-    <row r="2" spans="1:4" ht="30">
+    <row r="2" spans="1:4" ht="32">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1321,7 +1321,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="15">
+    <row r="12" spans="1:4" ht="16">
       <c r="A12" s="1" t="s">
         <v>26</v>
       </c>
@@ -1329,7 +1329,7 @@
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
     </row>
-    <row r="13" spans="1:4" ht="15">
+    <row r="13" spans="1:4" ht="16">
       <c r="A13" s="1" t="s">
         <v>27</v>
       </c>
@@ -1396,7 +1396,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -1409,7 +1409,7 @@
     <col min="10" max="10" width="5.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30">
+    <row r="1" spans="1:10" ht="32">
       <c r="A1" s="1" t="s">
         <v>41</v>
       </c>
@@ -3369,7 +3369,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -3385,7 +3385,7 @@
     <col min="16" max="16" width="9.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="30">
+    <row r="1" spans="1:16" ht="32">
       <c r="A1" s="1" t="s">
         <v>43</v>
       </c>
@@ -3943,7 +3943,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:Q14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.6640625" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -3953,7 +3953,7 @@
     <col min="17" max="17" width="11.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="30">
+    <row r="1" spans="1:17" ht="32">
       <c r="A1" s="1" t="s">
         <v>171</v>
       </c>
@@ -4703,7 +4703,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:S54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -4716,50 +4716,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="40" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="40" t="s">
         <v>193</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="34"/>
-      <c r="M1" s="34"/>
-      <c r="N1" s="34"/>
-      <c r="O1" s="34"/>
-      <c r="P1" s="34"/>
-      <c r="Q1" s="34"/>
-      <c r="R1" s="34"/>
-      <c r="S1" s="34"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
+      <c r="P1" s="40"/>
+      <c r="Q1" s="40"/>
+      <c r="R1" s="40"/>
+      <c r="S1" s="40"/>
     </row>
     <row r="2" spans="1:19" ht="29.25" customHeight="1">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="41" t="s">
         <v>194</v>
       </c>
-      <c r="B2" s="35"/>
-      <c r="C2" s="35"/>
-      <c r="D2" s="35"/>
-      <c r="E2" s="35"/>
-      <c r="F2" s="35"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
+      <c r="Q2" s="42"/>
+      <c r="R2" s="42"/>
+      <c r="S2" s="42"/>
     </row>
     <row r="3" spans="1:19">
       <c r="G3" s="5"/>
@@ -4777,75 +4777,75 @@
       <c r="S3" s="5"/>
     </row>
     <row r="4" spans="1:19" ht="34.75" customHeight="1">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="43" t="s">
         <v>195</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="37" t="s">
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43" t="s">
         <v>196</v>
       </c>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="38" t="s">
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="44" t="s">
         <v>197</v>
       </c>
-      <c r="H4" s="38"/>
-      <c r="I4" s="38"/>
-      <c r="J4" s="38" t="s">
+      <c r="H4" s="44"/>
+      <c r="I4" s="44"/>
+      <c r="J4" s="44" t="s">
         <v>198</v>
       </c>
-      <c r="K4" s="38"/>
-      <c r="L4" s="38"/>
-      <c r="M4" s="38" t="s">
+      <c r="K4" s="44"/>
+      <c r="L4" s="44"/>
+      <c r="M4" s="44" t="s">
         <v>199</v>
       </c>
-      <c r="N4" s="38"/>
-      <c r="O4" s="38"/>
-      <c r="P4" s="38" t="s">
+      <c r="N4" s="44"/>
+      <c r="O4" s="44"/>
+      <c r="P4" s="44" t="s">
         <v>200</v>
       </c>
-      <c r="Q4" s="38"/>
-      <c r="R4" s="38"/>
-      <c r="S4" s="38"/>
+      <c r="Q4" s="44"/>
+      <c r="R4" s="44"/>
+      <c r="S4" s="44"/>
     </row>
     <row r="5" spans="1:19" ht="37.25" customHeight="1">
-      <c r="A5" s="39">
+      <c r="A5" s="37">
         <f>SUMIF($E$10:$E$54,"Quantité exportée",$S$10:$S$54)</f>
         <v>3160.98</v>
       </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="40"/>
-      <c r="D5" s="41">
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="39">
         <f>SUMIF($E$10:$E$54,"Chiffre d'affaires MGA",$S$10:$S$54)</f>
         <v>19024357328</v>
       </c>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="41">
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="39">
         <f>SUMIFS($S$10:$S$54,$A$10:$A$54,"Japon",$E$10:$E$54,"Chiffre d'affaires MGA")</f>
         <v>5885836491</v>
       </c>
-      <c r="H5" s="42"/>
-      <c r="I5" s="42"/>
-      <c r="J5" s="41">
+      <c r="H5" s="34"/>
+      <c r="I5" s="34"/>
+      <c r="J5" s="39">
         <f>SUMIFS($S$10:$S$54,$A$10:$A$54,"Russie",$E$10:$E$54,"Chiffre d'affaires MGA")</f>
         <v>6497377284</v>
       </c>
-      <c r="K5" s="42"/>
-      <c r="L5" s="42"/>
-      <c r="M5" s="41">
+      <c r="K5" s="34"/>
+      <c r="L5" s="34"/>
+      <c r="M5" s="39">
         <f>SUMIFS($S$10:$S$54,$A$10:$A$54,"Chine",$E$10:$E$54,"Chiffre d'affaires MGA")</f>
         <v>6641143553</v>
       </c>
-      <c r="N5" s="42"/>
-      <c r="O5" s="42"/>
-      <c r="P5" s="42" t="s">
+      <c r="N5" s="34"/>
+      <c r="O5" s="34"/>
+      <c r="P5" s="34" t="s">
         <v>201</v>
       </c>
-      <c r="Q5" s="42"/>
-      <c r="R5" s="42"/>
-      <c r="S5" s="42"/>
+      <c r="Q5" s="34"/>
+      <c r="R5" s="34"/>
+      <c r="S5" s="34"/>
     </row>
     <row r="6" spans="1:19">
       <c r="G6" s="5"/>
@@ -4863,27 +4863,27 @@
       <c r="S6" s="5"/>
     </row>
     <row r="7" spans="1:19" ht="29.25" customHeight="1">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="35" t="s">
         <v>202</v>
       </c>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
-      <c r="G7" s="44"/>
-      <c r="H7" s="44"/>
-      <c r="I7" s="44"/>
-      <c r="J7" s="44"/>
-      <c r="K7" s="44"/>
-      <c r="L7" s="44"/>
-      <c r="M7" s="44"/>
-      <c r="N7" s="44"/>
-      <c r="O7" s="44"/>
-      <c r="P7" s="44"/>
-      <c r="Q7" s="44"/>
-      <c r="R7" s="44"/>
-      <c r="S7" s="44"/>
+      <c r="B7" s="35"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="36"/>
+      <c r="K7" s="36"/>
+      <c r="L7" s="36"/>
+      <c r="M7" s="36"/>
+      <c r="N7" s="36"/>
+      <c r="O7" s="36"/>
+      <c r="P7" s="36"/>
+      <c r="Q7" s="36"/>
+      <c r="R7" s="36"/>
+      <c r="S7" s="36"/>
     </row>
     <row r="8" spans="1:19">
       <c r="G8" s="5"/>
@@ -7616,13 +7616,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="P5:S5"/>
-    <mergeCell ref="A7:S7"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="M5:O5"/>
     <mergeCell ref="A1:S1"/>
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="A4:C4"/>
@@ -7631,6 +7624,13 @@
     <mergeCell ref="J4:L4"/>
     <mergeCell ref="M4:O4"/>
     <mergeCell ref="P4:S4"/>
+    <mergeCell ref="P5:S5"/>
+    <mergeCell ref="A7:S7"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="J5:L5"/>
+    <mergeCell ref="M5:O5"/>
   </mergeCells>
   <conditionalFormatting sqref="S10:S54">
     <cfRule type="dataBar" priority="1">
@@ -7677,7 +7677,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:Q19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5.1640625" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -7687,7 +7687,7 @@
     <col min="17" max="17" width="9.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="30">
+    <row r="1" spans="1:17" ht="32">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -8702,15 +8702,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:O7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
     <col min="2" max="2" width="4.6640625" customWidth="1"/>
-    <col min="3" max="14" width="11.1640625" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" customWidth="1"/>
+    <col min="4" max="14" width="11.1640625" customWidth="1"/>
     <col min="15" max="15" width="12.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="30">
+    <row r="1" spans="1:15" ht="32">
       <c r="A1" s="1" t="s">
         <v>203</v>
       </c>

</xml_diff>